<commit_message>
Add intraday monitor and update readme
</commit_message>
<xml_diff>
--- a/monitor_xlsx/20260302.xlsx
+++ b/monitor_xlsx/20260302.xlsx
@@ -94,8 +94,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -734,7 +734,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>111.43%</t>
+          <t>133.33%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -1204,18 +1204,31 @@
           <t>0050</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="G4" s="6" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>80.34999999999999</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="F4" t="n">
+        <v>224651</v>
+      </c>
+      <c r="G4" s="7" t="n">
         <v>-101500</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>-153600</v>
       </c>
       <c r="I4" t="n">
         <v>3214</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>30200</v>
       </c>
       <c r="K4" t="n">
         <v>54837</v>
@@ -1224,14 +1237,17 @@
         <v>8643</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>39383</v>
       </c>
       <c r="N4" t="n">
         <v>-4134246</v>
       </c>
+      <c r="O4" t="n">
+        <v>1.39</v>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏空</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1252,11 +1268,11 @@
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>-967</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -1268,14 +1284,14 @@
         <v>9643</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>49034</v>
       </c>
       <c r="N5" t="n">
         <v>-27513</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1295,18 +1311,31 @@
           <t>華城</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="G6" s="6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1030</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-3.74</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3792</v>
+      </c>
+      <c r="G6" s="7" t="n">
         <v>-723</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>3870</v>
       </c>
       <c r="I6" t="n">
         <v>39</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>-898</v>
       </c>
       <c r="K6" t="n">
         <v>173</v>
@@ -1315,11 +1344,14 @@
         <v>2936</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>14736</v>
       </c>
       <c r="N6" t="n">
         <v>-78749</v>
       </c>
+      <c r="O6" t="n">
+        <v>2.81</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>中性</t>
@@ -1342,18 +1374,31 @@
           <t>台達電</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="G7" s="7" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1425</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15569</v>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>210</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>3451</v>
       </c>
       <c r="I7" t="n">
         <v>162</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>3170</v>
       </c>
       <c r="K7" t="n">
         <v>337</v>
@@ -1362,14 +1407,17 @@
         <v>6395</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>32825</v>
       </c>
       <c r="N7" t="n">
         <v>-648849</v>
       </c>
+      <c r="O7" t="n">
+        <v>4.55</v>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1389,18 +1437,31 @@
           <t>台積電</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="G8" s="6" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1975</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>57404</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <v>-19539</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>-37942</v>
       </c>
       <c r="I8" t="n">
         <v>2624</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>8894</v>
       </c>
       <c r="K8" t="n">
         <v>1215</v>
@@ -1409,14 +1470,17 @@
         <v>22619</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>108149</v>
       </c>
       <c r="N8" t="n">
         <v>-6482919</v>
       </c>
+      <c r="O8" t="n">
+        <v>0.87</v>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏空</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1436,18 +1500,31 @@
           <t>華邦電</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="G9" s="7" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>124.5</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F9" t="n">
+        <v>155981</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>22448</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>26982</v>
       </c>
       <c r="I9" t="n">
         <v>951</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>25238</v>
       </c>
       <c r="K9" t="n">
         <v>1504</v>
@@ -1456,14 +1533,17 @@
         <v>132443</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>690462</v>
       </c>
       <c r="N9" t="n">
         <v>-1111395</v>
       </c>
+      <c r="O9" t="n">
+        <v>6.78</v>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1483,18 +1563,31 @@
           <t>台光電</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="G10" s="7" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2380</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3331</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>182</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-1656</v>
       </c>
       <c r="I10" t="n">
         <v>102</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="K10" t="n">
         <v>157</v>
@@ -1503,14 +1596,17 @@
         <v>1965</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>10930</v>
       </c>
       <c r="N10" t="n">
         <v>-89480</v>
       </c>
+      <c r="O10" t="n">
+        <v>3.12</v>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏空</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1530,18 +1626,31 @@
           <t>世芯-KY</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="G11" s="7" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3440</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1581</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>125</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>698</v>
       </c>
       <c r="I11" t="n">
         <v>-22</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="K11" t="n">
         <v>90</v>
@@ -1550,14 +1659,17 @@
         <v>5771</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>29259</v>
       </c>
       <c r="N11" t="n">
         <v>-19715</v>
       </c>
+      <c r="O11" t="n">
+        <v>0.53</v>
+      </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1577,18 +1689,31 @@
           <t>光聖</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="G12" s="6" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2355</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3957</v>
+      </c>
+      <c r="G12" s="7" t="n">
         <v>-608</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I12" t="n">
         <v>590</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="K12" t="n">
         <v>66</v>
@@ -1597,14 +1722,17 @@
         <v>4474</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>20998</v>
       </c>
       <c r="N12" t="n">
         <v>-19080</v>
       </c>
+      <c r="O12" t="n">
+        <v>14.99</v>
+      </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1624,18 +1752,31 @@
           <t>聯亞</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="G13" s="7" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>上櫃</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1390</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>-5.76</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6399</v>
+      </c>
+      <c r="G13" s="6" t="n">
         <v>132</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>-466</v>
       </c>
       <c r="I13" t="n">
         <v>143</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>-22</v>
       </c>
       <c r="K13" t="n">
         <v>10</v>
@@ -1644,14 +1785,17 @@
         <v>122</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>-223</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏空</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1671,18 +1815,31 @@
           <t>威剛</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="G14" s="6" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>上櫃</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>262</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="F14" t="n">
+        <v>16580</v>
+      </c>
+      <c r="G14" s="7" t="n">
         <v>-355</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>-9540</v>
       </c>
       <c r="I14" t="n">
         <v>-441</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>-3468</v>
       </c>
       <c r="K14" t="n">
         <v>454</v>
@@ -1691,14 +1848,17 @@
         <v>96</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>487</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>主力積極賣出</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -1718,18 +1878,31 @@
           <t>台新科</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="G15" s="6" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>上櫃</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>127</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>-9.609999999999999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2433</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>-544</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>989</v>
       </c>
       <c r="I15" t="n">
         <v>-1</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="K15" t="n">
         <v>-151</v>
@@ -1738,11 +1911,14 @@
         <v>95</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
       <c r="P15" t="inlineStr">
         <is>
           <t>中性</t>
@@ -1765,18 +1941,31 @@
           <t>華星光</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="G16" s="7" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>上櫃</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>418.5</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>-9.9</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4583</v>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>963</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I16" t="n">
         <v>1179</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>2798</v>
       </c>
       <c r="K16" t="n">
         <v>-57</v>
@@ -1785,14 +1974,17 @@
         <v>-322</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>-1527</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>主力積極買進</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -1812,18 +2004,31 @@
           <t>景碩</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="G17" s="6" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>304.5</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>-3.18</v>
+      </c>
+      <c r="F17" t="n">
+        <v>41298</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>-3998</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>-1341</v>
       </c>
       <c r="I17" t="n">
         <v>-113</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1995</v>
       </c>
       <c r="K17" t="n">
         <v>1261</v>
@@ -1832,14 +2037,17 @@
         <v>19539</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>98779</v>
       </c>
       <c r="N17" t="n">
         <v>-113508</v>
       </c>
+      <c r="O17" t="n">
+        <v>0.26</v>
+      </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏空</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -1859,12 +2067,25 @@
           <t>耀登</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="G18" s="7" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>217.5</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="F18" t="n">
+        <v>6384</v>
+      </c>
+      <c r="G18" s="6" t="n">
         <v>278</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>-347</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1876,14 +2097,17 @@
         <v>5601</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>22351</v>
       </c>
       <c r="N18" t="n">
         <v>-11200</v>
       </c>
+      <c r="O18" t="n">
+        <v>23.16</v>
+      </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>主力積極賣出</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">

</xml_diff>